<commit_message>
Ajustando o documento xlsx e definindo a média
</commit_message>
<xml_diff>
--- a/notas4B.xlsx
+++ b/notas4B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\Pipline-Leitura-de-Notas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E8CE2C4-F2B7-442C-9076-A5663C0CA2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00F3FF94-A97F-4263-BB60-861487C96E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1068,9 +1068,9 @@
         <f t="shared" ref="J7:J36" si="0">H7/I7</f>
         <v>6.625</v>
       </c>
-      <c r="K7" s="33" t="str">
-        <f>IF(ROUND(J7,0)&lt;=6, ROUND(J7,0)&amp;" - Reprovado", ROUND(J7,0)&amp;" - Aprovado")</f>
-        <v>7 - Aprovado</v>
+      <c r="K7" s="33">
+        <f>ROUND(VALUE(J7),0)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1">
@@ -1106,9 +1106,9 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K8" s="33" t="str">
-        <f t="shared" ref="K8:K36" si="1">IF(ROUND(J8,0)&lt;=6, ROUND(J8,0)&amp;" - Reprovado", ROUND(J8,0)&amp;" - Aprovado")</f>
-        <v>5 - Reprovado</v>
+      <c r="K8" s="33">
+        <f t="shared" ref="K8:K36" si="1">ROUND(VALUE(J8),0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1">
@@ -1144,9 +1144,9 @@
         <f t="shared" si="0"/>
         <v>6.25</v>
       </c>
-      <c r="K9" s="33" t="str">
+      <c r="K9" s="33">
         <f t="shared" si="1"/>
-        <v>6 - Reprovado</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1">
@@ -1182,9 +1182,9 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="K10" s="33" t="str">
+      <c r="K10" s="33">
         <f t="shared" si="1"/>
-        <v>7 - Aprovado</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1">
@@ -1220,9 +1220,9 @@
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
-      <c r="K11" s="33" t="str">
+      <c r="K11" s="33">
         <f t="shared" si="1"/>
-        <v>5 - Reprovado</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="14.25" customHeight="1">
@@ -1258,9 +1258,9 @@
         <f t="shared" si="0"/>
         <v>8.75</v>
       </c>
-      <c r="K12" s="33" t="str">
+      <c r="K12" s="33">
         <f t="shared" si="1"/>
-        <v>9 - Aprovado</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="14.25" customHeight="1">
@@ -1296,9 +1296,9 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="K13" s="33" t="str">
+      <c r="K13" s="33">
         <f t="shared" si="1"/>
-        <v>6 - Reprovado</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="14.25" customHeight="1">
@@ -1334,9 +1334,9 @@
         <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
-      <c r="K14" s="33" t="str">
+      <c r="K14" s="33">
         <f t="shared" si="1"/>
-        <v>9 - Aprovado</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="14.25" customHeight="1">
@@ -1372,9 +1372,9 @@
         <f t="shared" si="0"/>
         <v>9.25</v>
       </c>
-      <c r="K15" s="33" t="str">
+      <c r="K15" s="33">
         <f t="shared" si="1"/>
-        <v>9 - Aprovado</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="14.25" customHeight="1">
@@ -1410,9 +1410,9 @@
         <f t="shared" si="0"/>
         <v>7.85</v>
       </c>
-      <c r="K16" s="33" t="str">
+      <c r="K16" s="33">
         <f t="shared" si="1"/>
-        <v>8 - Aprovado</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="14.25" customHeight="1">
@@ -1448,9 +1448,9 @@
         <f t="shared" si="0"/>
         <v>6.75</v>
       </c>
-      <c r="K17" s="33" t="str">
+      <c r="K17" s="33">
         <f t="shared" si="1"/>
-        <v>7 - Aprovado</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="14.25" customHeight="1">
@@ -1486,9 +1486,9 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="K18" s="33" t="str">
+      <c r="K18" s="33">
         <f t="shared" si="1"/>
-        <v>3 - Reprovado</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="14.25" customHeight="1">
@@ -1524,9 +1524,9 @@
         <f t="shared" si="0"/>
         <v>3.25</v>
       </c>
-      <c r="K19" s="33" t="str">
+      <c r="K19" s="33">
         <f t="shared" si="1"/>
-        <v>3 - Reprovado</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="14.25" customHeight="1">
@@ -1562,9 +1562,9 @@
         <f t="shared" si="0"/>
         <v>1.625</v>
       </c>
-      <c r="K20" s="33" t="str">
+      <c r="K20" s="33">
         <f t="shared" si="1"/>
-        <v>2 - Reprovado</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="14.25" customHeight="1">
@@ -1600,9 +1600,9 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="K21" s="33" t="str">
+      <c r="K21" s="33">
         <f t="shared" si="1"/>
-        <v>3 - Reprovado</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="14.25" customHeight="1">
@@ -1638,9 +1638,9 @@
         <f t="shared" si="0"/>
         <v>5.25</v>
       </c>
-      <c r="K22" s="33" t="str">
+      <c r="K22" s="33">
         <f t="shared" si="1"/>
-        <v>5 - Reprovado</v>
+        <v>5</v>
       </c>
       <c r="L22" s="2"/>
     </row>
@@ -1677,9 +1677,9 @@
         <f t="shared" si="0"/>
         <v>9.75</v>
       </c>
-      <c r="K23" s="33" t="str">
+      <c r="K23" s="33">
         <f t="shared" si="1"/>
-        <v>10 - Aprovado</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="14.25" customHeight="1">
@@ -1715,9 +1715,9 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="K24" s="33" t="str">
+      <c r="K24" s="33">
         <f t="shared" si="1"/>
-        <v>7 - Aprovado</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="14.25" customHeight="1">
@@ -1753,9 +1753,9 @@
         <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
-      <c r="K25" s="33" t="str">
+      <c r="K25" s="33">
         <f t="shared" si="1"/>
-        <v>9 - Aprovado</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="14.25" customHeight="1">
@@ -1791,9 +1791,9 @@
         <f t="shared" si="0"/>
         <v>4.75</v>
       </c>
-      <c r="K26" s="33" t="str">
+      <c r="K26" s="33">
         <f t="shared" si="1"/>
-        <v>5 - Reprovado</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="14.25" customHeight="1">
@@ -1829,9 +1829,9 @@
         <f t="shared" si="0"/>
         <v>4.1500000000000004</v>
       </c>
-      <c r="K27" s="33" t="str">
+      <c r="K27" s="33">
         <f t="shared" si="1"/>
-        <v>4 - Reprovado</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="14.25" customHeight="1">
@@ -1867,9 +1867,9 @@
         <f t="shared" si="0"/>
         <v>8.25</v>
       </c>
-      <c r="K28" s="33" t="str">
+      <c r="K28" s="33">
         <f t="shared" si="1"/>
-        <v>8 - Aprovado</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="14.25" customHeight="1">
@@ -1905,9 +1905,9 @@
         <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
-      <c r="K29" s="33" t="str">
+      <c r="K29" s="33">
         <f t="shared" si="1"/>
-        <v>10 - Aprovado</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="14.25" customHeight="1">
@@ -1943,9 +1943,9 @@
         <f t="shared" si="0"/>
         <v>9.75</v>
       </c>
-      <c r="K30" s="33" t="str">
+      <c r="K30" s="33">
         <f t="shared" si="1"/>
-        <v>10 - Aprovado</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="14.25" customHeight="1">
@@ -1981,9 +1981,9 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="K31" s="33" t="str">
+      <c r="K31" s="33">
         <f t="shared" si="1"/>
-        <v>3 - Reprovado</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="14.25" customHeight="1">
@@ -2019,9 +2019,9 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="K32" s="33" t="str">
+      <c r="K32" s="33">
         <f t="shared" si="1"/>
-        <v>3 - Reprovado</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="14.25" customHeight="1">
@@ -2057,9 +2057,9 @@
         <f t="shared" si="0"/>
         <v>8.875</v>
       </c>
-      <c r="K33" s="33" t="str">
+      <c r="K33" s="33">
         <f t="shared" si="1"/>
-        <v>9 - Aprovado</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="14.25" customHeight="1">
@@ -2095,9 +2095,9 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="K34" s="33" t="str">
+      <c r="K34" s="33">
         <f t="shared" si="1"/>
-        <v>7 - Aprovado</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="14.25" customHeight="1">
@@ -2133,9 +2133,9 @@
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
-      <c r="K35" s="33" t="str">
+      <c r="K35" s="33">
         <f t="shared" si="1"/>
-        <v>5 - Reprovado</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="14.25" customHeight="1">
@@ -2171,9 +2171,9 @@
         <f t="shared" si="0"/>
         <v>8.25</v>
       </c>
-      <c r="K36" s="33" t="str">
+      <c r="K36" s="33">
         <f t="shared" si="1"/>
-        <v>8 - Aprovado</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="14.25" customHeight="1">

</xml_diff>